<commit_message>
Strip company-name prefixes/suffixes from 7 restaurant names
(주)엔바이콘 하이포크/아시안퀴진똠/하림닭요리/순우가/왕스덕/교소바 -> drop
the "(주)엔바이콘 " prefix; 강창구찹쌀진순대 판교테크원점(유한회사 이로) ->
drop the trailing legal-entity suffix. Updates the bundled source xlsx
and seed-data.json to stay in sync with the live renamed list.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wmp-restaurant/scripts/source-data/restaurants.xlsx
+++ b/wmp-restaurant/scripts/source-data/restaurants.xlsx
@@ -709,7 +709,7 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>강창구찹쌀진순대 판교테크원점(유한회사 이로)</v>
+        <v>강창구찹쌀진순대 판교테크원점</v>
       </c>
       <c r="B29" t="str">
         <v>13529) 경기도 성남시 분당구 분당내곡로 131 지하1층 27호</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>(주)엔바이콘 하이포크</v>
+        <v>하이포크</v>
       </c>
       <c r="B73" t="str">
         <v>13487) 경기도 성남시 분당구 대왕판교로645번길 36</v>
@@ -1270,7 +1270,7 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>(주)엔바이콘 아시안퀴진똠</v>
+        <v>아시안퀴진똠</v>
       </c>
       <c r="B80" t="str">
         <v>13487) 경기 성남시 분당구 대왕판교로645번길 36 삼평동</v>
@@ -1556,7 +1556,7 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>(주)엔바이콘 하림닭요리</v>
+        <v>하림닭요리</v>
       </c>
       <c r="B106" t="str">
         <v>13487) 경기도 성남시 분당구 대왕판교로645번길 36</v>
@@ -2458,7 +2458,7 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>(주)엔바이콘 순우가</v>
+        <v>순우가</v>
       </c>
       <c r="B188" t="str">
         <v>13487) 경기도 성남시 분당구 대왕판교로645번길 36</v>
@@ -2843,7 +2843,7 @@
     </row>
     <row r="223">
       <c r="A223" t="str">
-        <v>(주)엔바이콘 왕스덕</v>
+        <v>왕스덕</v>
       </c>
       <c r="B223" t="str">
         <v>13487) 경기도 성남시 분당구 대왕판교로645번길 36</v>
@@ -2964,7 +2964,7 @@
     </row>
     <row r="234">
       <c r="A234" t="str">
-        <v>(주)엔바이콘 교소바</v>
+        <v>교소바</v>
       </c>
       <c r="B234" t="str">
         <v>13487) 경기도 성남시 분당구 대왕판교로645번길 36 NS홈쇼핑 지하1층</v>

</xml_diff>